<commit_message>
Actualizar catalogo a Tarifas 2026 con selector de Tarifa (PVP / T1) y simplificar a confeccion de facturas
</commit_message>
<xml_diff>
--- a/registro_compras_ventas.xlsx
+++ b/registro_compras_ventas.xlsx
@@ -56,7 +56,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>21/08/2026</t>
+          <t>22/08/2026</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -168,7 +168,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>21/08/2026</t>
+          <t>22/08/2026</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">

</xml_diff>